<commit_message>
Full update of all project Excel files with corrected exact floor parsing
</commit_message>
<xml_diff>
--- a/files/九龙-何文田-傲玟.xlsx
+++ b/files/九龙-何文田-傲玟.xlsx
@@ -27626,10 +27626,34 @@
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr"/>
+      <c r="C6" s="22" t="inlineStr">
+        <is>
+          <t>B | 1442呎 (1房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="inlineStr">
+        <is>
+          <t>C | 1251呎 (3房)
+-
+-
+(待售)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
           <t>27&amp;28&amp;29</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>A | 6681呎 (4+房)
 -
@@ -27637,32 +27661,8 @@
 (待售)</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr"/>
-      <c r="D6" s="20" t="inlineStr"/>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr"/>
-      <c r="C7" s="22" t="inlineStr">
-        <is>
-          <t>B | 1442呎 (1房)
--
--
-(待售)</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>C | 1251呎 (3房)
--
--
-(待售)</t>
-        </is>
-      </c>
+      <c r="C7" s="20" t="inlineStr"/>
+      <c r="D7" s="20" t="inlineStr"/>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -28476,10 +28476,34 @@
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="inlineStr"/>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>B | 1351呎 (3房)
+$3630万
+$26,866/呎
+(24年-04月-24日)</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="inlineStr">
+        <is>
+          <t>C | 1180呎 (3房)
+$2612万
+$22,139/呎
+(25年-09月-12日)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
           <t>27&amp;28</t>
         </is>
       </c>
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
         <is>
           <t>A | 2338呎 (4+房)
 $7600万
@@ -28487,32 +28511,8 @@
 (24年-04月-09日)</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr"/>
-      <c r="D6" s="20" t="inlineStr"/>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="B7" s="20" t="inlineStr"/>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>B | 1351呎 (3房)
-$3630万
-$26,866/呎
-(24年-04月-24日)</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>C | 1180呎 (3房)
-$2612万
-$22,139/呎
-(25年-09月-12日)</t>
-        </is>
-      </c>
+      <c r="C7" s="20" t="inlineStr"/>
+      <c r="D7" s="20" t="inlineStr"/>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -29326,12 +29326,30 @@
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
+          <t>28&amp;29</t>
+        </is>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>A | 3255呎 (4+房)
+$11039万
+$33,915/呎
+(25年-02月-26日)</t>
+        </is>
+      </c>
+      <c r="C6" s="20" t="inlineStr"/>
+      <c r="D6" s="20" t="inlineStr"/>
+      <c r="E6" s="20" t="inlineStr"/>
+    </row>
+    <row r="7" ht="58" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr"/>
-      <c r="C6" s="20" t="inlineStr"/>
-      <c r="D6" s="21" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr"/>
+      <c r="C7" s="20" t="inlineStr"/>
+      <c r="D7" s="21" t="inlineStr">
         <is>
           <t>C | 845呎 (2房)
 $1984万
@@ -29339,7 +29357,7 @@
 (25年-03月-11日)</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="E7" s="21" t="inlineStr">
         <is>
           <t>D | 845呎 (2房)
 $1873万
@@ -29347,24 +29365,6 @@
 (25年-07月-11日)</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>28&amp;29</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>A | 3255呎 (4+房)
-$11039万
-$33,915/呎
-(25年-02月-26日)</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr"/>
-      <c r="D7" s="20" t="inlineStr"/>
-      <c r="E7" s="20" t="inlineStr"/>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -31148,11 +31148,29 @@
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
         <is>
+          <t>19&amp;20</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>A | 2258呎 (4+房)
+$7128万
+$31,568/呎
+(26年-01月-27日)</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr"/>
+      <c r="D8" s="20" t="inlineStr"/>
+      <c r="E8" s="20" t="inlineStr"/>
+    </row>
+    <row r="9" ht="58" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr"/>
-      <c r="C8" s="21" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr"/>
+      <c r="C9" s="21" t="inlineStr">
         <is>
           <t>B | 1264呎 (3房)
 $3021万
@@ -31160,7 +31178,7 @@
 (25年-10月-08日)</t>
         </is>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D9" s="21" t="inlineStr">
         <is>
           <t>C | 808呎 (2房)
 $1912万
@@ -31168,7 +31186,7 @@
 (24年-03月-22日)</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="E9" s="21" t="inlineStr">
         <is>
           <t>D | 808呎 (2房)
 $1916万
@@ -31176,24 +31194,6 @@
 (24年-01月-12日)</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
-        <is>
-          <t>19&amp;20</t>
-        </is>
-      </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>A | 2258呎 (4+房)
-$7128万
-$31,568/呎
-(26年-01月-27日)</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr"/>
-      <c r="D9" s="20" t="inlineStr"/>
-      <c r="E9" s="20" t="inlineStr"/>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="19" t="inlineStr">

</xml_diff>